<commit_message>
Versao 27.0  -  Correcao de mesclagem
</commit_message>
<xml_diff>
--- a/pacientes.xlsx
+++ b/pacientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa de Automatizacao Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73DF62B1-F832-4E7B-8119-A22BA4208635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1D068E-B28B-46FE-AE07-933514DD1D06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="300">
   <si>
     <t>ENFERMARIA</t>
   </si>
@@ -44,40 +44,67 @@
     <t>OBSERVAÇÕES</t>
   </si>
   <si>
+    <t>Apartamento 01</t>
+  </si>
+  <si>
+    <t>Ana Clara</t>
+  </si>
+  <si>
+    <t>Hipossódica</t>
+  </si>
+  <si>
+    <t>Monitorar pressão arterial diariamente.</t>
+  </si>
+  <si>
     <t>Apartamento 02</t>
   </si>
   <si>
     <t>401</t>
   </si>
   <si>
-    <t>FULANO</t>
-  </si>
-  <si>
-    <t>PASTOSA + HAS</t>
+    <t>Carlos Oliveira</t>
+  </si>
+  <si>
+    <t>Diabética</t>
+  </si>
+  <si>
+    <t>Evitar frutas com alto índice glicêmico à noite.</t>
   </si>
   <si>
     <t>402</t>
   </si>
   <si>
+    <t>Mariana Santos</t>
+  </si>
+  <si>
+    <t>Low Carb</t>
+  </si>
+  <si>
+    <t>Aumentar ingestão de fibras e água.</t>
+  </si>
+  <si>
     <t>403</t>
   </si>
   <si>
-    <t>JOÃOZINHO</t>
-  </si>
-  <si>
-    <t>BRANDA+HAS</t>
-  </si>
-  <si>
-    <t>S/FEIJÃO E S/FRANGO</t>
+    <t>Pedro Souza</t>
+  </si>
+  <si>
+    <t>Hiperproteica</t>
+  </si>
+  <si>
+    <t>Foco em recuperação muscular pós-treino.</t>
   </si>
   <si>
     <t>Apartamento 03</t>
   </si>
   <si>
-    <t>MARCELINHA</t>
-  </si>
-  <si>
-    <t>PARENTERAL</t>
+    <t>Beatriz Costa</t>
+  </si>
+  <si>
+    <t>Vegetariana</t>
+  </si>
+  <si>
+    <t>Suplementação de B12 recomendada.</t>
   </si>
   <si>
     <t>Cirurgica Extra</t>
@@ -86,344 +113,827 @@
     <t>701</t>
   </si>
   <si>
+    <t>João Pereira</t>
+  </si>
+  <si>
+    <t>Sem Glúten</t>
+  </si>
+  <si>
+    <t>Paciente com Doença Celíaca.</t>
+  </si>
+  <si>
     <t>702</t>
   </si>
   <si>
-    <t>PINOQUIO</t>
-  </si>
-  <si>
-    <t>LÍQUIDA PASTOSA</t>
+    <t>Fernanda Lima</t>
+  </si>
+  <si>
+    <t>Sem Lactose</t>
+  </si>
+  <si>
+    <t>Intolerância severa a lácteos.</t>
   </si>
   <si>
     <t>703</t>
   </si>
   <si>
-    <t>URSINHO POF</t>
-  </si>
-  <si>
-    <t>LÍQUIDA DE PROVA (100ml)</t>
+    <t>Ricardo Gomes</t>
+  </si>
+  <si>
+    <t>Cetogênica</t>
+  </si>
+  <si>
+    <t>Acompanhar função renal mensalmente.</t>
   </si>
   <si>
     <t>704</t>
   </si>
   <si>
-    <t>DONATELLO</t>
-  </si>
-  <si>
-    <t>BRANDA + DM</t>
+    <t>Camila Rocha</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Sem restrições alimentares conhecidas.</t>
   </si>
   <si>
     <t>705</t>
   </si>
   <si>
+    <t>Lucas Martins</t>
+  </si>
+  <si>
+    <t>Hipocalórica</t>
+  </si>
+  <si>
+    <t>Objetivo: perda de peso gradual (500g/semana).</t>
+  </si>
+  <si>
     <t>Pediatria</t>
   </si>
   <si>
     <t>801</t>
   </si>
   <si>
+    <t>Juliana Alves</t>
+  </si>
+  <si>
+    <t>Líquida Restrita</t>
+  </si>
+  <si>
+    <t>Pós-operatório imediato (24h).</t>
+  </si>
+  <si>
     <t>802</t>
   </si>
   <si>
+    <t>Gabriel Dias</t>
+  </si>
+  <si>
+    <t>Pastosa</t>
+  </si>
+  <si>
+    <t>Paciente com disfagia leve.</t>
+  </si>
+  <si>
     <t>803</t>
   </si>
   <si>
+    <t>Patricia Barbosa</t>
+  </si>
+  <si>
+    <t>Rica em Ferro</t>
+  </si>
+  <si>
+    <t>Tratamento de anemia ferropriva.</t>
+  </si>
+  <si>
     <t>804</t>
   </si>
   <si>
-    <t>DOMINIC TORETTO</t>
-  </si>
-  <si>
-    <t>PARA IDADE (1A E 1M)</t>
-  </si>
-  <si>
-    <t>LEITE APTAMIL PEPTI, ACEITA FRANGO AO MOLHO</t>
+    <t>Rafael Ferreira</t>
+  </si>
+  <si>
+    <t>Mediterrânea</t>
+  </si>
+  <si>
+    <t>Prevenção cardiovascular.</t>
   </si>
   <si>
     <t>805</t>
   </si>
   <si>
-    <t>BRIAN COONER</t>
-  </si>
-  <si>
-    <t>PARA IDADE (5 ANOS)</t>
-  </si>
-  <si>
-    <t>S/LACTOSE + RH (ACEITA FRUTAS E FRANGO ASSADO)</t>
+    <t>Sofia Rodrigues</t>
+  </si>
+  <si>
+    <t>DASH</t>
+  </si>
+  <si>
+    <t>Controle de hipertensão arterial.</t>
   </si>
   <si>
     <t>806</t>
   </si>
   <si>
+    <t>Roberto Almeida</t>
+  </si>
+  <si>
+    <t>Renal Crônica</t>
+  </si>
+  <si>
+    <t>Restrição severa de potássio e fósforo.</t>
+  </si>
+  <si>
     <t>Enfermaria Masculina</t>
   </si>
   <si>
     <t>901</t>
   </si>
   <si>
-    <t>OPTIMUS PRIME</t>
-  </si>
-  <si>
-    <t>LIVRE + LAXATIVA</t>
-  </si>
-  <si>
-    <t>SEM SOPA</t>
+    <t>Vanessa Moreira</t>
+  </si>
+  <si>
+    <t>Low FODMAP</t>
+  </si>
+  <si>
+    <t>Síndrome do Intestino Irritável (fase de eliminação).</t>
   </si>
   <si>
     <t>902</t>
   </si>
   <si>
+    <t>Daniel Carvalho</t>
+  </si>
+  <si>
+    <t>Hipercalórica</t>
+  </si>
+  <si>
+    <t>Suporte nutricional para paciente oncológico.</t>
+  </si>
+  <si>
     <t>903</t>
   </si>
   <si>
-    <t>LUFFY</t>
-  </si>
-  <si>
-    <t>BRANDA + HIPERPROTEICA + HAS + RH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FRUTAS MOLES </t>
+    <t>Eliane Pinto</t>
+  </si>
+  <si>
+    <t>Branda</t>
+  </si>
+  <si>
+    <t>Gastrite crônica; evitar irritantes gástricos.</t>
   </si>
   <si>
     <t>904</t>
   </si>
   <si>
+    <t>Thiago Mendes</t>
+  </si>
+  <si>
+    <t>Sem Frutos do Mar</t>
+  </si>
+  <si>
+    <t>Alergia grave (risco de choque anafilático).</t>
+  </si>
+  <si>
     <t>905</t>
   </si>
   <si>
+    <t>Larissa Azevedo</t>
+  </si>
+  <si>
+    <t>Vegana</t>
+  </si>
+  <si>
+    <t>Monitorar níveis de ferro e ferritina.</t>
+  </si>
+  <si>
     <t>906</t>
   </si>
   <si>
+    <t>Bruno Nogueira</t>
+  </si>
+  <si>
+    <t>Leve</t>
+  </si>
+  <si>
+    <t>Pós-operatório tardio de vesícula.</t>
+  </si>
+  <si>
     <t>907</t>
   </si>
   <si>
+    <t>Carla Ribeiro</t>
+  </si>
+  <si>
+    <t>Hipolipídica</t>
+  </si>
+  <si>
+    <t>Controle rigoroso de triglicerídeos.</t>
+  </si>
+  <si>
     <t>Enfermaria Femenina</t>
   </si>
   <si>
     <t>1001</t>
   </si>
   <si>
+    <t>Felipe Castro</t>
+  </si>
+  <si>
+    <t>Sem Oleaginosas</t>
+  </si>
+  <si>
+    <t>Alergia a amendoim e castanhas.</t>
+  </si>
+  <si>
     <t>1002</t>
   </si>
   <si>
+    <t>Amanda Correia</t>
+  </si>
+  <si>
+    <t>Rica em Fibras</t>
+  </si>
+  <si>
+    <t>Tratamento para constipação crônica.</t>
+  </si>
+  <si>
     <t>1003</t>
   </si>
   <si>
+    <t>Gustavo Farias</t>
+  </si>
+  <si>
+    <t>Líquida Completa</t>
+  </si>
+  <si>
+    <t>Preparação para exame de colonoscopia.</t>
+  </si>
+  <si>
     <t>1004</t>
   </si>
   <si>
+    <t>Helena Vieira</t>
+  </si>
+  <si>
+    <t>Controle de Vitamina K</t>
+  </si>
+  <si>
+    <t>Paciente em uso de anticoagulante (Varfarina).</t>
+  </si>
+  <si>
     <t>1005</t>
   </si>
   <si>
+    <t>André Ramos</t>
+  </si>
+  <si>
+    <t>Pastosa Homogênea</t>
+  </si>
+  <si>
+    <t>Alto risco de broncoaspiração (idoso).</t>
+  </si>
+  <si>
     <t>1006</t>
   </si>
   <si>
+    <t>Monica Teixeira</t>
+  </si>
+  <si>
+    <t>Sem Açúcar</t>
+  </si>
+  <si>
+    <t>Diabetes Gestacional (monitorar glicemia).</t>
+  </si>
+  <si>
     <t>1007</t>
   </si>
   <si>
+    <t>Rodrigo Santana</t>
+  </si>
+  <si>
+    <t>Rica em Cálcio</t>
+  </si>
+  <si>
+    <t>Diagnóstico recente de osteoporose.</t>
+  </si>
+  <si>
     <t>Maternidade Normal</t>
   </si>
   <si>
     <t>301</t>
   </si>
   <si>
+    <t>Leticia Guimarães</t>
+  </si>
+  <si>
+    <t>Anti-inflamatória</t>
+  </si>
+  <si>
+    <t>Auxílio no tratamento de artrite reumatoide.</t>
+  </si>
+  <si>
     <t>302</t>
   </si>
   <si>
+    <t>Marcelo Cruz</t>
+  </si>
+  <si>
+    <t>Pobre em Purinas</t>
+  </si>
+  <si>
+    <t>Crise aguda de Gota (evitar carnes vermelhas).</t>
+  </si>
+  <si>
     <t>303</t>
   </si>
   <si>
+    <t>Renata Lopes</t>
+  </si>
+  <si>
+    <t>Sem Soja</t>
+  </si>
+  <si>
+    <t>Intolerância alimentar específica.</t>
+  </si>
+  <si>
     <t>304</t>
   </si>
   <si>
+    <t>Vitor Campos</t>
+  </si>
+  <si>
+    <t>Bariátrica (Fase 3)</t>
+  </si>
+  <si>
+    <t>Introdução de alimentos sólidos bem mastigados.</t>
+  </si>
+  <si>
     <t>Maternidade Cesárea</t>
   </si>
   <si>
     <t>201</t>
   </si>
   <si>
-    <t>MAGALI</t>
+    <t>Cintia Duarte</t>
+  </si>
+  <si>
+    <t>Pediátrica Geral</t>
+  </si>
+  <si>
+    <t>Acompanhamento de introdução alimentar (6 meses).</t>
+  </si>
+  <si>
+    <t>202</t>
+  </si>
+  <si>
+    <t>Paulo Azevedo</t>
+  </si>
+  <si>
+    <t>Cicatrização de úlcera de pressão (escaras).</t>
+  </si>
+  <si>
+    <t>203</t>
+  </si>
+  <si>
+    <t>Jessica Lima</t>
+  </si>
+  <si>
+    <t>Sensibilidade não celíaca ao glúten.</t>
+  </si>
+  <si>
+    <t>204</t>
+  </si>
+  <si>
+    <t>Diego Torres</t>
+  </si>
+  <si>
+    <t>Controle de crises epilépticas refratárias.</t>
+  </si>
+  <si>
+    <t>205</t>
+  </si>
+  <si>
+    <t>Simone Vieira</t>
+  </si>
+  <si>
+    <t>Restrição Hídrica</t>
+  </si>
+  <si>
+    <t>Insuficiência cardíaca congestiva (max 1L/dia).</t>
+  </si>
+  <si>
+    <t>206</t>
+  </si>
+  <si>
+    <t>Renato Mendes</t>
+  </si>
+  <si>
+    <t>Hipossódica Leve</t>
+  </si>
+  <si>
+    <t>Prevenção primária (histórico familiar de HAS).</t>
+  </si>
+  <si>
+    <t>207</t>
+  </si>
+  <si>
+    <t>Tatiana Cunha</t>
+  </si>
+  <si>
+    <t>Enteral (Sonda)</t>
+  </si>
+  <si>
+    <t>Dieta polimérica padrão (1.5 kcal/ml).</t>
+  </si>
+  <si>
+    <t>208</t>
+  </si>
+  <si>
+    <t>Igor Vasconcelos</t>
+  </si>
+  <si>
+    <t>Desconforto abdominal e gases após ingestão.</t>
+  </si>
+  <si>
+    <t>209</t>
+  </si>
+  <si>
+    <t>Cláudia Ramos</t>
+  </si>
+  <si>
+    <t>Controle de colesterol LDL alto.</t>
+  </si>
+  <si>
+    <t>210</t>
+  </si>
+  <si>
+    <t>Fabio Junior</t>
+  </si>
+  <si>
+    <t>Sem Cítricos</t>
+  </si>
+  <si>
+    <t>Refluxo gastroesofágico grave (evitar acidez).</t>
+  </si>
+  <si>
+    <t>Cirúgica Feminina</t>
+  </si>
+  <si>
+    <t>501</t>
+  </si>
+  <si>
+    <t>Alice Batista</t>
+  </si>
+  <si>
+    <t>Líquida Clara</t>
+  </si>
+  <si>
+    <t>Preparo pré-operatório (cirurgia gástrica).</t>
+  </si>
+  <si>
+    <t>502</t>
+  </si>
+  <si>
+    <t>Hugo Almeida</t>
+  </si>
+  <si>
+    <t>Sem Ovos</t>
+  </si>
+  <si>
+    <t>Alergia mediada por IgE (excluir traços).</t>
+  </si>
+  <si>
+    <t>503</t>
+  </si>
+  <si>
+    <t>Debora Santos</t>
+  </si>
+  <si>
+    <t>Controle de resistência à insulina.</t>
+  </si>
+  <si>
+    <t>504</t>
+  </si>
+  <si>
+    <t>Sergio Molina</t>
+  </si>
+  <si>
+    <t>Recuperação de gastroenterite viral.</t>
+  </si>
+  <si>
+    <t>505</t>
+  </si>
+  <si>
+    <t>Luana Pires</t>
+  </si>
+  <si>
+    <t>Ganho de peso (IMC &lt; 18.5).</t>
+  </si>
+  <si>
+    <t>506</t>
+  </si>
+  <si>
+    <t>Matheus Silva</t>
+  </si>
+  <si>
+    <t>Sem Cafeína</t>
+  </si>
+  <si>
+    <t>Tratamento de ansiedade severa e insônia.</t>
+  </si>
+  <si>
+    <t>Cirúgica Masculina</t>
+  </si>
+  <si>
+    <t>101</t>
+  </si>
+  <si>
+    <t>Elisa Fogo</t>
+  </si>
+  <si>
+    <t>Sem Tiramina</t>
+  </si>
+  <si>
+    <t>Uso de inibidores da MAO (antidepressivos).</t>
+  </si>
+  <si>
+    <t>102</t>
+  </si>
+  <si>
+    <t>Caio Ribeiro</t>
+  </si>
+  <si>
+    <t>Pobre em Oxalato</t>
+  </si>
+  <si>
+    <t>Prevenção de cálculos renais recorrentes.</t>
+  </si>
+  <si>
+    <t>103</t>
+  </si>
+  <si>
+    <t>Vera Lúcia</t>
+  </si>
+  <si>
+    <t>Rica em Potássio</t>
+  </si>
+  <si>
+    <t>Uso de diuréticos espoliadores de K+.</t>
+  </si>
+  <si>
+    <t>104</t>
+  </si>
+  <si>
+    <t>Otávio Neto</t>
+  </si>
+  <si>
+    <t>Sem Corantes</t>
+  </si>
+  <si>
+    <t>Alergia a tartrazina (amarelo crepúsculo).</t>
+  </si>
+  <si>
+    <t>105</t>
+  </si>
+  <si>
+    <t>Gisele Bueno</t>
+  </si>
+  <si>
+    <t>Vegetariana Estrita</t>
+  </si>
+  <si>
+    <t>Opção ética; monitorar ingestão proteica.</t>
+  </si>
+  <si>
+    <t>106</t>
+  </si>
+  <si>
+    <t>Leonardo Paz</t>
+  </si>
+  <si>
+    <t>Sem Sementes</t>
+  </si>
+  <si>
+    <t>Diverticulite (fase de remissão).</t>
+  </si>
+  <si>
+    <t>Pré-Parto</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Maraiza Costa</t>
+  </si>
+  <si>
+    <t>Parenteral</t>
+  </si>
+  <si>
+    <t>Síndrome do Intestino Curto (nutrição venosa).</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Nivaldo Filho</t>
+  </si>
+  <si>
+    <t>Sem Histamina</t>
+  </si>
+  <si>
+    <t>Intolerância à histamina (evitar fermentados).</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Paloma Siqueira</t>
+  </si>
+  <si>
+    <t>Hipoglicídica</t>
+  </si>
+  <si>
+    <t>Pré-diabetes (foco em carboidratos complexos).</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Samuel Borges</t>
+  </si>
+  <si>
+    <t>Sem Sulfito</t>
+  </si>
+  <si>
+    <t>Asma induzida por sulfitos (vinho/frutas secas).</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Talita Nunes</t>
+  </si>
+  <si>
+    <t>Rica em Zinco</t>
+  </si>
+  <si>
+    <t>Fortalecimento do sistema imune pós-infecção.</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Vicente Paulo</t>
+  </si>
+  <si>
+    <t>Sem Carne Vermelha</t>
+  </si>
+  <si>
+    <t>Dislipidemia mista e digestão lenta.</t>
+  </si>
+  <si>
+    <t>Breno Koster</t>
+  </si>
+  <si>
+    <t>Líquida Fria</t>
+  </si>
+  <si>
+    <t>Pós-operatório de amigdalectomia (evitar sangramento).</t>
+  </si>
+  <si>
+    <t>Iara Souza</t>
+  </si>
+  <si>
+    <t>Sem Frituras</t>
+  </si>
+  <si>
+    <t>Dislipidemia grave; preferir grelhados e assados.</t>
+  </si>
+  <si>
+    <t>Kleber Matos</t>
+  </si>
+  <si>
+    <t>Recuperação de grandes queimaduras (regeneração tecidual).</t>
+  </si>
+  <si>
+    <t>Ursula Viana</t>
+  </si>
+  <si>
+    <t>Cetogênica Cíclica</t>
+  </si>
+  <si>
+    <t>Protocolo esportivo para performance em endurance.</t>
+  </si>
+  <si>
+    <t>Wagner Lima</t>
+  </si>
+  <si>
+    <t>Hipolipídica Estrita</t>
+  </si>
+  <si>
+    <t>Pancreatite crônica (minimizar estímulo pancreático).</t>
+  </si>
+  <si>
+    <t>Ximena Luz</t>
+  </si>
+  <si>
+    <t>Sem Níquel</t>
+  </si>
+  <si>
+    <t>Dermatite de contato sistêmica (evitar cacau e aveia).</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Yasmin Flor</t>
+  </si>
+  <si>
+    <t>Rica em Ômega-3</t>
+  </si>
+  <si>
+    <t>Suporte nutricional neurológico e anti-inflamatório.</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>Zeca Ferreira</t>
+  </si>
+  <si>
+    <t>Controle de Ácido Úrico</t>
+  </si>
+  <si>
+    <t>Prevenção de crises de gota; hidratação intensa.</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>Quezia Dantas</t>
+  </si>
+  <si>
+    <t>Branda Mecânica</t>
+  </si>
+  <si>
+    <t>Dificuldade de mastigação (adaptação de prótese dentária).</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Valter Lins</t>
+  </si>
+  <si>
+    <t>Sem Fenilalanina</t>
+  </si>
+  <si>
+    <t>Fenilcetonúria (PKU) - monitoramento rigoroso.</t>
+  </si>
+  <si>
+    <t>ESTAB 01</t>
+  </si>
+  <si>
+    <t>MICHAEL</t>
+  </si>
+  <si>
+    <t>LIQUIDA</t>
+  </si>
+  <si>
+    <t>ESTAB 02</t>
+  </si>
+  <si>
+    <t>TREVOR</t>
+  </si>
+  <si>
+    <t>PASTOSA</t>
+  </si>
+  <si>
+    <t>ESTAB 03</t>
+  </si>
+  <si>
+    <t>FRANKLIN</t>
   </si>
   <si>
     <t>LIVRE</t>
   </si>
   <si>
-    <t>202</t>
-  </si>
-  <si>
-    <t>MÔNICA</t>
-  </si>
-  <si>
-    <t>S/SOPA</t>
-  </si>
-  <si>
-    <t>203</t>
-  </si>
-  <si>
-    <t>204</t>
-  </si>
-  <si>
-    <t>205</t>
-  </si>
-  <si>
-    <t>206</t>
-  </si>
-  <si>
-    <t>207</t>
-  </si>
-  <si>
-    <t>208</t>
-  </si>
-  <si>
-    <t>209</t>
-  </si>
-  <si>
-    <t>210</t>
-  </si>
-  <si>
-    <t>Cirúgica Feminina</t>
-  </si>
-  <si>
-    <t>501</t>
-  </si>
-  <si>
-    <t>VELMA</t>
-  </si>
-  <si>
-    <t>502</t>
-  </si>
-  <si>
-    <t>DAPHINY</t>
-  </si>
-  <si>
-    <t>503</t>
-  </si>
-  <si>
-    <t>504</t>
-  </si>
-  <si>
-    <t>505</t>
-  </si>
-  <si>
-    <t>506</t>
-  </si>
-  <si>
-    <t>Cirúgica Masculina</t>
-  </si>
-  <si>
-    <t>101</t>
-  </si>
-  <si>
-    <t>SALSICHA</t>
-  </si>
-  <si>
-    <t>S/BISCOITO SCOOBY</t>
-  </si>
-  <si>
-    <t>102</t>
-  </si>
-  <si>
-    <t>FRED</t>
-  </si>
-  <si>
-    <t>PASTOSA(200ml)</t>
-  </si>
-  <si>
-    <t>103</t>
-  </si>
-  <si>
-    <t>TITIO AVÔ</t>
-  </si>
-  <si>
-    <t>104</t>
-  </si>
-  <si>
-    <t>105</t>
-  </si>
-  <si>
-    <t>106</t>
-  </si>
-  <si>
-    <t>Pré-Parto</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>REBECA</t>
-  </si>
-  <si>
-    <t>PASTOSA</t>
-  </si>
-  <si>
-    <t>ESSA OBS É UM TESTE DE PRODUÇÃO</t>
-  </si>
-  <si>
-    <t>AUGUSTO CARRARA DE SOSUA</t>
-  </si>
-  <si>
-    <t>LIQUIDA</t>
-  </si>
-  <si>
-    <t>MORANGUINHO</t>
-  </si>
-  <si>
-    <t>ESSA OBS É UM TESTE DE PRODUÇÃO PODE E DEVE SER APAGADO</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>ESTAB 01</t>
-  </si>
-  <si>
-    <t>MICHAEL</t>
-  </si>
-  <si>
-    <t>ESTAB 02</t>
-  </si>
-  <si>
-    <t>TREVOR</t>
-  </si>
-  <si>
-    <t>ESTAB 03</t>
-  </si>
-  <si>
-    <t>FRANKLIN</t>
-  </si>
-  <si>
-    <t>Apartamento 01</t>
+    <t>EXTRA</t>
+  </si>
+  <si>
+    <t>Fabio Cruz</t>
+  </si>
+  <si>
+    <t>Sem Sopa</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -435,11 +945,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -477,16 +982,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -790,10 +1289,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -814,614 +1317,1065 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>41</v>
+      </c>
+      <c r="E10" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>48</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>52</v>
+      </c>
+      <c r="C13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="E15" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>68</v>
+      </c>
+      <c r="C17" t="s">
+        <v>69</v>
+      </c>
+      <c r="D17" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="D18" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="E18" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="B19" t="s">
-        <v>47</v>
+        <v>77</v>
+      </c>
+      <c r="C19" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="B20" t="s">
-        <v>48</v>
+        <v>81</v>
       </c>
       <c r="C20" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
       <c r="D20" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="E20" t="s">
-        <v>51</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>85</v>
+      </c>
+      <c r="C21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>89</v>
+      </c>
+      <c r="C22" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" t="s">
+        <v>91</v>
+      </c>
+      <c r="E22" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>93</v>
+      </c>
+      <c r="C23" t="s">
+        <v>94</v>
+      </c>
+      <c r="D23" t="s">
+        <v>95</v>
+      </c>
+      <c r="E23" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>97</v>
+      </c>
+      <c r="C24" t="s">
+        <v>98</v>
+      </c>
+      <c r="D24" t="s">
+        <v>99</v>
+      </c>
+      <c r="E24" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>102</v>
+      </c>
+      <c r="C25" t="s">
+        <v>103</v>
+      </c>
+      <c r="D25" t="s">
+        <v>104</v>
+      </c>
+      <c r="E25" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="B26" t="s">
-        <v>58</v>
+        <v>106</v>
+      </c>
+      <c r="C26" t="s">
+        <v>107</v>
+      </c>
+      <c r="D26" t="s">
+        <v>108</v>
+      </c>
+      <c r="E26" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="B27" t="s">
-        <v>59</v>
+        <v>110</v>
+      </c>
+      <c r="C27" t="s">
+        <v>111</v>
+      </c>
+      <c r="D27" t="s">
+        <v>112</v>
+      </c>
+      <c r="E27" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
+        <v>114</v>
+      </c>
+      <c r="C28" t="s">
+        <v>115</v>
+      </c>
+      <c r="D28" t="s">
+        <v>116</v>
+      </c>
+      <c r="E28" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="B29" t="s">
-        <v>61</v>
+        <v>118</v>
+      </c>
+      <c r="C29" t="s">
+        <v>119</v>
+      </c>
+      <c r="D29" t="s">
+        <v>120</v>
+      </c>
+      <c r="E29" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>122</v>
+      </c>
+      <c r="C30" t="s">
+        <v>123</v>
+      </c>
+      <c r="D30" t="s">
+        <v>124</v>
+      </c>
+      <c r="E30" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="B31" t="s">
-        <v>63</v>
+        <v>126</v>
+      </c>
+      <c r="C31" t="s">
+        <v>127</v>
+      </c>
+      <c r="D31" t="s">
+        <v>128</v>
+      </c>
+      <c r="E31" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>64</v>
+        <v>130</v>
       </c>
       <c r="B32" t="s">
-        <v>65</v>
+        <v>131</v>
+      </c>
+      <c r="C32" t="s">
+        <v>132</v>
+      </c>
+      <c r="D32" t="s">
+        <v>133</v>
+      </c>
+      <c r="E32" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>64</v>
+        <v>130</v>
       </c>
       <c r="B33" t="s">
-        <v>66</v>
+        <v>135</v>
+      </c>
+      <c r="C33" t="s">
+        <v>136</v>
+      </c>
+      <c r="D33" t="s">
+        <v>137</v>
+      </c>
+      <c r="E33" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>64</v>
+        <v>130</v>
       </c>
       <c r="B34" t="s">
-        <v>67</v>
+        <v>139</v>
+      </c>
+      <c r="C34" t="s">
+        <v>140</v>
+      </c>
+      <c r="D34" t="s">
+        <v>141</v>
+      </c>
+      <c r="E34" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>64</v>
+        <v>130</v>
       </c>
       <c r="B35" t="s">
-        <v>68</v>
+        <v>143</v>
+      </c>
+      <c r="C35" t="s">
+        <v>144</v>
+      </c>
+      <c r="D35" t="s">
+        <v>145</v>
+      </c>
+      <c r="E35" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="B36" t="s">
-        <v>70</v>
+        <v>148</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>149</v>
       </c>
       <c r="D36" t="s">
-        <v>72</v>
+        <v>150</v>
+      </c>
+      <c r="E36" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="B37" t="s">
-        <v>73</v>
+        <v>152</v>
       </c>
       <c r="C37" t="s">
-        <v>74</v>
+        <v>153</v>
       </c>
       <c r="D37" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>75</v>
+        <v>154</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>155</v>
+      </c>
+      <c r="C38" t="s">
+        <v>156</v>
+      </c>
+      <c r="D38" t="s">
+        <v>29</v>
+      </c>
+      <c r="E38" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="B39" t="s">
-        <v>77</v>
+        <v>158</v>
+      </c>
+      <c r="C39" t="s">
+        <v>159</v>
+      </c>
+      <c r="D39" t="s">
+        <v>37</v>
+      </c>
+      <c r="E39" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="B40" t="s">
-        <v>78</v>
+        <v>161</v>
+      </c>
+      <c r="C40" t="s">
+        <v>162</v>
+      </c>
+      <c r="D40" t="s">
+        <v>163</v>
+      </c>
+      <c r="E40" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="B41" t="s">
-        <v>79</v>
+        <v>165</v>
+      </c>
+      <c r="C41" t="s">
+        <v>166</v>
+      </c>
+      <c r="D41" t="s">
+        <v>167</v>
+      </c>
+      <c r="E41" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="B42" t="s">
-        <v>80</v>
+        <v>169</v>
+      </c>
+      <c r="C42" t="s">
+        <v>170</v>
+      </c>
+      <c r="D42" t="s">
+        <v>171</v>
+      </c>
+      <c r="E42" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="B43" t="s">
-        <v>81</v>
+        <v>173</v>
+      </c>
+      <c r="C43" t="s">
+        <v>174</v>
+      </c>
+      <c r="D43" t="s">
+        <v>33</v>
+      </c>
+      <c r="E43" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="B44" t="s">
-        <v>82</v>
+        <v>176</v>
+      </c>
+      <c r="C44" t="s">
+        <v>177</v>
+      </c>
+      <c r="D44" t="s">
+        <v>108</v>
+      </c>
+      <c r="E44" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="B45" t="s">
-        <v>83</v>
+        <v>179</v>
+      </c>
+      <c r="C45" t="s">
+        <v>180</v>
+      </c>
+      <c r="D45" t="s">
+        <v>181</v>
+      </c>
+      <c r="E45" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>84</v>
+        <v>183</v>
       </c>
       <c r="B46" t="s">
-        <v>85</v>
+        <v>184</v>
       </c>
       <c r="C46" t="s">
-        <v>86</v>
+        <v>185</v>
+      </c>
+      <c r="D46" t="s">
+        <v>186</v>
+      </c>
+      <c r="E46" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>84</v>
+        <v>183</v>
       </c>
       <c r="B47" t="s">
-        <v>87</v>
+        <v>188</v>
       </c>
       <c r="C47" t="s">
-        <v>88</v>
+        <v>189</v>
+      </c>
+      <c r="D47" t="s">
+        <v>190</v>
+      </c>
+      <c r="E47" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>84</v>
+        <v>183</v>
       </c>
       <c r="B48" t="s">
-        <v>89</v>
+        <v>192</v>
+      </c>
+      <c r="C48" t="s">
+        <v>193</v>
+      </c>
+      <c r="D48" t="s">
+        <v>16</v>
+      </c>
+      <c r="E48" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>84</v>
+        <v>183</v>
       </c>
       <c r="B49" t="s">
-        <v>90</v>
+        <v>195</v>
+      </c>
+      <c r="C49" t="s">
+        <v>196</v>
+      </c>
+      <c r="D49" t="s">
+        <v>83</v>
+      </c>
+      <c r="E49" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>84</v>
+        <v>183</v>
       </c>
       <c r="B50" t="s">
-        <v>91</v>
+        <v>198</v>
+      </c>
+      <c r="C50" t="s">
+        <v>199</v>
+      </c>
+      <c r="D50" t="s">
+        <v>79</v>
+      </c>
+      <c r="E50" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>84</v>
+        <v>183</v>
       </c>
       <c r="B51" t="s">
-        <v>92</v>
+        <v>201</v>
+      </c>
+      <c r="C51" t="s">
+        <v>202</v>
+      </c>
+      <c r="D51" t="s">
+        <v>203</v>
+      </c>
+      <c r="E51" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>93</v>
+        <v>205</v>
       </c>
       <c r="B52" t="s">
-        <v>94</v>
+        <v>206</v>
       </c>
       <c r="C52" t="s">
-        <v>95</v>
+        <v>207</v>
       </c>
       <c r="D52" t="s">
-        <v>72</v>
+        <v>208</v>
       </c>
       <c r="E52" t="s">
-        <v>96</v>
+        <v>209</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>93</v>
+        <v>205</v>
       </c>
       <c r="B53" t="s">
-        <v>97</v>
+        <v>210</v>
       </c>
       <c r="C53" t="s">
-        <v>98</v>
+        <v>211</v>
       </c>
       <c r="D53" t="s">
-        <v>99</v>
+        <v>212</v>
+      </c>
+      <c r="E53" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>93</v>
+        <v>205</v>
       </c>
       <c r="B54" t="s">
-        <v>100</v>
+        <v>214</v>
       </c>
       <c r="C54" t="s">
-        <v>101</v>
+        <v>215</v>
       </c>
       <c r="D54" t="s">
-        <v>50</v>
+        <v>216</v>
+      </c>
+      <c r="E54" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>93</v>
+        <v>205</v>
       </c>
       <c r="B55" t="s">
-        <v>102</v>
+        <v>218</v>
+      </c>
+      <c r="C55" t="s">
+        <v>219</v>
+      </c>
+      <c r="D55" t="s">
+        <v>220</v>
+      </c>
+      <c r="E55" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>93</v>
+        <v>205</v>
       </c>
       <c r="B56" t="s">
-        <v>103</v>
+        <v>222</v>
+      </c>
+      <c r="C56" t="s">
+        <v>223</v>
+      </c>
+      <c r="D56" t="s">
+        <v>224</v>
+      </c>
+      <c r="E56" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>93</v>
+        <v>205</v>
       </c>
       <c r="B57" t="s">
-        <v>104</v>
+        <v>226</v>
+      </c>
+      <c r="C57" t="s">
+        <v>227</v>
+      </c>
+      <c r="D57" t="s">
+        <v>228</v>
+      </c>
+      <c r="E57" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>105</v>
+        <v>205</v>
       </c>
       <c r="B58" t="s">
-        <v>106</v>
+        <v>297</v>
+      </c>
+      <c r="C58" t="s">
+        <v>298</v>
+      </c>
+      <c r="D58" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>105</v>
+        <v>230</v>
       </c>
       <c r="B59" t="s">
-        <v>107</v>
+        <v>231</v>
+      </c>
+      <c r="C59" t="s">
+        <v>232</v>
+      </c>
+      <c r="D59" t="s">
+        <v>233</v>
+      </c>
+      <c r="E59" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>105</v>
+        <v>230</v>
       </c>
       <c r="B60" t="s">
-        <v>108</v>
+        <v>235</v>
+      </c>
+      <c r="C60" t="s">
+        <v>236</v>
+      </c>
+      <c r="D60" t="s">
+        <v>237</v>
+      </c>
+      <c r="E60" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>105</v>
+        <v>230</v>
       </c>
       <c r="B61" t="s">
-        <v>109</v>
+        <v>239</v>
+      </c>
+      <c r="C61" t="s">
+        <v>240</v>
+      </c>
+      <c r="D61" t="s">
+        <v>241</v>
+      </c>
+      <c r="E61" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>105</v>
+        <v>230</v>
       </c>
       <c r="B62" t="s">
-        <v>110</v>
+        <v>243</v>
+      </c>
+      <c r="C62" t="s">
+        <v>244</v>
+      </c>
+      <c r="D62" t="s">
+        <v>245</v>
+      </c>
+      <c r="E62" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>105</v>
+        <v>230</v>
       </c>
       <c r="B63" t="s">
-        <v>111</v>
+        <v>247</v>
+      </c>
+      <c r="C63" t="s">
+        <v>248</v>
+      </c>
+      <c r="D63" t="s">
+        <v>249</v>
+      </c>
+      <c r="E63" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>230</v>
+      </c>
+      <c r="B64" t="s">
+        <v>251</v>
+      </c>
+      <c r="C64" t="s">
+        <v>252</v>
+      </c>
+      <c r="D64" t="s">
+        <v>253</v>
+      </c>
+      <c r="E64" t="s">
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -1450,79 +2404,142 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>231</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>255</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>256</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>235</v>
       </c>
       <c r="B3" t="s">
-        <v>115</v>
+        <v>258</v>
       </c>
       <c r="C3" t="s">
-        <v>116</v>
+        <v>259</v>
       </c>
       <c r="D3" t="s">
-        <v>114</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>108</v>
+        <v>239</v>
       </c>
       <c r="B4" t="s">
-        <v>117</v>
+        <v>261</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>118</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>243</v>
+      </c>
+      <c r="B5" t="s">
+        <v>263</v>
+      </c>
+      <c r="C5" t="s">
+        <v>264</v>
+      </c>
+      <c r="D5" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>110</v>
+        <v>247</v>
+      </c>
+      <c r="B6" t="s">
+        <v>266</v>
+      </c>
+      <c r="C6" t="s">
+        <v>267</v>
+      </c>
+      <c r="D6" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>111</v>
+        <v>251</v>
+      </c>
+      <c r="B7" t="s">
+        <v>269</v>
+      </c>
+      <c r="C7" t="s">
+        <v>270</v>
+      </c>
+      <c r="D7" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>119</v>
+        <v>272</v>
+      </c>
+      <c r="B8" t="s">
+        <v>273</v>
+      </c>
+      <c r="C8" t="s">
+        <v>274</v>
+      </c>
+      <c r="D8" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>120</v>
+        <v>276</v>
+      </c>
+      <c r="B9" t="s">
+        <v>277</v>
+      </c>
+      <c r="C9" t="s">
+        <v>278</v>
+      </c>
+      <c r="D9" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>121</v>
+        <v>280</v>
+      </c>
+      <c r="B10" t="s">
+        <v>281</v>
+      </c>
+      <c r="C10" t="s">
+        <v>282</v>
+      </c>
+      <c r="D10" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>122</v>
+        <v>284</v>
+      </c>
+      <c r="B11" t="s">
+        <v>285</v>
+      </c>
+      <c r="C11" t="s">
+        <v>286</v>
+      </c>
+      <c r="D11" t="s">
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -1551,35 +2568,35 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>288</v>
       </c>
       <c r="B2" t="s">
-        <v>124</v>
+        <v>289</v>
       </c>
       <c r="C2" t="s">
-        <v>116</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>291</v>
       </c>
       <c r="B3" t="s">
-        <v>126</v>
+        <v>292</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>294</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
+        <v>295</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>